<commit_message>
adicionadas anotacoes aos plots
</commit_message>
<xml_diff>
--- a/base_consolidada.xlsx
+++ b/base_consolidada.xlsx
@@ -3,18 +3,19 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6322C3FB-8BEA-4950-BD26-F0D5F41D7128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0868636D-7982-4789-8B1E-3B976D75E630}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" firstSheet="6" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="regioes" sheetId="1" r:id="rId1"/>
     <sheet name="inadimplentes" sheetId="2" r:id="rId2"/>
     <sheet name="setores" sheetId="3" r:id="rId3"/>
     <sheet name="urbanizacao" sheetId="4" r:id="rId4"/>
-    <sheet name="custo_de_vida" sheetId="5" r:id="rId5"/>
-    <sheet name="populacao_por_regiao" sheetId="7" r:id="rId6"/>
-    <sheet name="populacao_por_estado" sheetId="6" r:id="rId7"/>
+    <sheet name="taxa_de_desemprego_SP" sheetId="8" r:id="rId5"/>
+    <sheet name="custo_de_vida" sheetId="5" r:id="rId6"/>
+    <sheet name="populacao_por_regiao" sheetId="7" r:id="rId7"/>
+    <sheet name="populacao_por_estado" sheetId="6" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7124" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7127" uniqueCount="98">
   <si>
     <t>mes</t>
   </si>
@@ -318,6 +319,15 @@
     <t>taxa_rural</t>
   </si>
   <si>
+    <t>ano</t>
+  </si>
+  <si>
+    <t>trimestre</t>
+  </si>
+  <si>
+    <t>taxa_de_desemprego</t>
+  </si>
+  <si>
     <t>custo_de_vida</t>
   </si>
   <si>
@@ -328,9 +338,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -365,7 +376,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -378,6 +389,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -89809,6 +89821,559 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{992B224D-4017-4EBD-9254-1B5154C2A7DB}">
+  <dimension ref="A1:C49"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="2" width="10.28515625" customWidth="1"/>
+    <col min="3" max="3" width="16.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2">
+        <v>2012</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="8">
+        <v>7.8E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3">
+        <v>2012</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3" s="8">
+        <v>7.4999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4">
+        <v>2012</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4" s="8">
+        <v>7.0000000000000007E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5">
+        <v>2012</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5" s="8">
+        <v>6.8000000000000005E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6">
+        <v>2013</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" s="8">
+        <v>7.8E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7">
+        <v>2013</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" s="8">
+        <v>7.4999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8">
+        <v>2013</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" s="8">
+        <v>7.3999999999999996E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9">
+        <v>2013</v>
+      </c>
+      <c r="B9">
+        <v>4</v>
+      </c>
+      <c r="C9" s="8">
+        <v>6.6000000000000003E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10">
+        <v>2014</v>
+      </c>
+      <c r="B10">
+        <v>1</v>
+      </c>
+      <c r="C10" s="8">
+        <v>7.2999999999999995E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11">
+        <v>2014</v>
+      </c>
+      <c r="B11">
+        <v>2</v>
+      </c>
+      <c r="C11" s="8">
+        <v>7.0999999999999994E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12">
+        <v>2014</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+      <c r="C12" s="8">
+        <v>7.2999999999999995E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13">
+        <v>2014</v>
+      </c>
+      <c r="B13">
+        <v>4</v>
+      </c>
+      <c r="C13" s="8">
+        <v>7.1999999999999995E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14">
+        <v>2015</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" s="8">
+        <v>8.5999999999999993E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15">
+        <v>2015</v>
+      </c>
+      <c r="B15">
+        <v>2</v>
+      </c>
+      <c r="C15" s="8">
+        <v>9.1999999999999998E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16">
+        <v>2015</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+      <c r="C16" s="8">
+        <v>9.8000000000000004E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17">
+        <v>2015</v>
+      </c>
+      <c r="B17">
+        <v>4</v>
+      </c>
+      <c r="C17" s="8">
+        <v>0.10199999999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18">
+        <v>2016</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18" s="8">
+        <v>0.122</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19">
+        <v>2016</v>
+      </c>
+      <c r="B19">
+        <v>2</v>
+      </c>
+      <c r="C19" s="8">
+        <v>0.123</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20">
+        <v>2016</v>
+      </c>
+      <c r="B20">
+        <v>3</v>
+      </c>
+      <c r="C20" s="8">
+        <v>0.129</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21">
+        <v>2016</v>
+      </c>
+      <c r="B21">
+        <v>4</v>
+      </c>
+      <c r="C21" s="8">
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22">
+        <v>2017</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22" s="8">
+        <v>0.14399999999999999</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23">
+        <v>2017</v>
+      </c>
+      <c r="B23">
+        <v>2</v>
+      </c>
+      <c r="C23" s="8">
+        <v>0.13600000000000001</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24">
+        <v>2017</v>
+      </c>
+      <c r="B24">
+        <v>3</v>
+      </c>
+      <c r="C24" s="8">
+        <v>0.13300000000000001</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25">
+        <v>2017</v>
+      </c>
+      <c r="B25">
+        <v>4</v>
+      </c>
+      <c r="C25" s="8">
+        <v>0.128</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26">
+        <v>2018</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26" s="8">
+        <v>0.14099999999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27">
+        <v>2018</v>
+      </c>
+      <c r="B27">
+        <v>2</v>
+      </c>
+      <c r="C27" s="8">
+        <v>0.13800000000000001</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28">
+        <v>2018</v>
+      </c>
+      <c r="B28">
+        <v>3</v>
+      </c>
+      <c r="C28" s="8">
+        <v>0.13300000000000001</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29">
+        <v>2018</v>
+      </c>
+      <c r="B29">
+        <v>4</v>
+      </c>
+      <c r="C29" s="8">
+        <v>0.126</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30">
+        <v>2019</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30" s="8">
+        <v>0.13600000000000001</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31">
+        <v>2019</v>
+      </c>
+      <c r="B31">
+        <v>2</v>
+      </c>
+      <c r="C31" s="8">
+        <v>0.129</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32">
+        <v>2019</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+      <c r="C32" s="8">
+        <v>0.122</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33">
+        <v>2019</v>
+      </c>
+      <c r="B33">
+        <v>4</v>
+      </c>
+      <c r="C33" s="8">
+        <v>0.11600000000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34">
+        <v>2020</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" s="8">
+        <v>0.123</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35">
+        <v>2022</v>
+      </c>
+      <c r="B35">
+        <v>2</v>
+      </c>
+      <c r="C35" s="8">
+        <v>9.1999999999999998E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36">
+        <v>2022</v>
+      </c>
+      <c r="B36">
+        <v>3</v>
+      </c>
+      <c r="C36" s="8">
+        <v>8.6999999999999994E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37">
+        <v>2022</v>
+      </c>
+      <c r="B37">
+        <v>4</v>
+      </c>
+      <c r="C37" s="8">
+        <v>7.6999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38">
+        <v>2023</v>
+      </c>
+      <c r="B38">
+        <v>1</v>
+      </c>
+      <c r="C38" s="8">
+        <v>8.5000000000000006E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39">
+        <v>2023</v>
+      </c>
+      <c r="B39">
+        <v>2</v>
+      </c>
+      <c r="C39" s="8">
+        <v>7.8E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40">
+        <v>2023</v>
+      </c>
+      <c r="B40">
+        <v>3</v>
+      </c>
+      <c r="C40" s="8">
+        <v>7.1999999999999995E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41">
+        <v>2023</v>
+      </c>
+      <c r="B41">
+        <v>4</v>
+      </c>
+      <c r="C41" s="8">
+        <v>6.9000000000000006E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
+      <c r="A42">
+        <v>2024</v>
+      </c>
+      <c r="B42">
+        <v>1</v>
+      </c>
+      <c r="C42" s="8">
+        <v>7.3999999999999996E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
+      <c r="A43">
+        <v>2024</v>
+      </c>
+      <c r="B43">
+        <v>2</v>
+      </c>
+      <c r="C43" s="8">
+        <v>6.4000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
+      <c r="A44">
+        <v>2024</v>
+      </c>
+      <c r="B44">
+        <v>3</v>
+      </c>
+      <c r="C44" s="8">
+        <v>6.0999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45">
+        <v>2024</v>
+      </c>
+      <c r="B45">
+        <v>4</v>
+      </c>
+      <c r="C45" s="8">
+        <v>5.8999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46">
+        <v>2025</v>
+      </c>
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="C46" s="8">
+        <v>6.3E-2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47">
+        <v>2025</v>
+      </c>
+      <c r="B47">
+        <v>2</v>
+      </c>
+      <c r="C47" s="8">
+        <v>5.0999999999999997E-2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48">
+        <v>2025</v>
+      </c>
+      <c r="B48">
+        <v>3</v>
+      </c>
+      <c r="C48" s="8">
+        <v>5.1999999999999998E-2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49">
+        <v>2025</v>
+      </c>
+      <c r="B49">
+        <v>4</v>
+      </c>
+      <c r="C49" s="8">
+        <v>4.7E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A13C640D-86CB-4947-AA6A-D8DE9BCC57F6}">
   <dimension ref="A1:C28"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -89826,7 +90391,7 @@
         <v>9</v>
       </c>
       <c r="C1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -90131,7 +90696,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2DD8842-429E-4698-971E-E17066B3382D}">
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -90145,7 +90710,7 @@
         <v>10</v>
       </c>
       <c r="B1" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -90193,7 +90758,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92E26E54-D99D-40F9-8644-54D789936BB2}">
   <dimension ref="A1:B28"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -90207,7 +90772,7 @@
         <v>8</v>
       </c>
       <c r="B1" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:2">

</xml_diff>